<commit_message>
Fill equipment ledger with data extracted from uploaded documents
Populate first row of the registration ledger with the mobile crane
(KATO SL-600II) details extracted from the uploaded registration
certificate, insurance policy, operator license, and business
registration PDF.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011AyaoccyvsKxVgYNBrnxVL
</commit_message>
<xml_diff>
--- a/output/건설기계_기초자료_관리대장.xlsx
+++ b/output/건설기계_기초자료_관리대장.xlsx
@@ -70,7 +70,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -92,11 +92,55 @@
         <color rgb="00B7B7B7"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -123,6 +167,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -197,6 +243,26 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="J6" authorId="0" shapeId="0">
+      <text>
+        <t>업로드된 서류(사업자등록증·보험증권·등록증)에서 소유자(중앙크레인/김효영) 연락처를 찾지 못해 공란 처리했습니다.</t>
+      </text>
+    </comment>
+    <comment ref="L6" authorId="0" shapeId="0">
+      <text>
+        <t>등록·검사증 뒷면 손글씨 기재분으로 판독이 어려워 추정 입력했습니다. 원본 서류로 반드시 재확인 바랍니다.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -535,47 +601,47 @@
           <t>기본정보</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
+      <c r="B3" s="10" t="n"/>
+      <c r="C3" s="10" t="n"/>
+      <c r="D3" s="10" t="n"/>
+      <c r="E3" s="10" t="n"/>
+      <c r="F3" s="10" t="n"/>
+      <c r="G3" s="11" t="n"/>
       <c r="H3" s="3" t="inlineStr">
         <is>
           <t>소유/연락처</t>
         </is>
       </c>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="n"/>
+      <c r="I3" s="10" t="n"/>
+      <c r="J3" s="11" t="n"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
           <t>검사현황</t>
         </is>
       </c>
-      <c r="L3" s="4" t="n"/>
+      <c r="L3" s="11" t="n"/>
       <c r="M3" s="3" t="inlineStr">
         <is>
           <t>보험현황</t>
         </is>
       </c>
-      <c r="N3" s="4" t="n"/>
-      <c r="O3" s="4" t="n"/>
+      <c r="N3" s="10" t="n"/>
+      <c r="O3" s="11" t="n"/>
       <c r="P3" s="3" t="inlineStr">
         <is>
           <t>운전원정보</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="n"/>
-      <c r="R3" s="4" t="n"/>
-      <c r="S3" s="4" t="n"/>
+      <c r="Q3" s="10" t="n"/>
+      <c r="R3" s="10" t="n"/>
+      <c r="S3" s="11" t="n"/>
       <c r="T3" s="3" t="inlineStr">
         <is>
           <t>현장정보</t>
         </is>
       </c>
-      <c r="U3" s="4" t="n"/>
-      <c r="V3" s="4" t="n"/>
+      <c r="U3" s="10" t="n"/>
+      <c r="V3" s="11" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -801,27 +867,109 @@
       <c r="A6" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
-      <c r="L6" s="8" t="n"/>
-      <c r="M6" s="8" t="n"/>
-      <c r="N6" s="8" t="n"/>
-      <c r="O6" s="8" t="n"/>
-      <c r="P6" s="8" t="n"/>
-      <c r="Q6" s="8" t="n"/>
-      <c r="R6" s="8" t="n"/>
-      <c r="S6" s="8" t="n"/>
-      <c r="T6" s="9" t="n"/>
-      <c r="U6" s="9" t="n"/>
-      <c r="V6" s="8" t="n"/>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>이동식크레인(라프터크레인)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>SL-600Ⅱ(KR-50H-L2) / 51톤</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>대전007가8717</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>KR512-2074</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>KATO(가토)</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>2006</v>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>중앙크레인</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>김효영</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>정기검사</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>2025-01-22 ~ 2026-02-02</t>
+        </is>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>삼성화재해상보험(주)</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>125E0476450000</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>2025-03-03 ~ 2026-03-03</t>
+        </is>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>정철훈</t>
+        </is>
+      </c>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t>기중기(이동식크레인)·지게차</t>
+        </is>
+      </c>
+      <c r="R6" s="8" t="inlineStr">
+        <is>
+          <t>대전20-2013-0057-00</t>
+        </is>
+      </c>
+      <c r="S6" s="8" t="inlineStr">
+        <is>
+          <t>2025-12-31(안전교육 기준, 취득 2013-05-16)</t>
+        </is>
+      </c>
+      <c r="T6" s="9" t="inlineStr">
+        <is>
+          <t>청사동 중앙홀(단열공사)</t>
+        </is>
+      </c>
+      <c r="U6" s="8" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="V6" s="9" t="inlineStr">
+        <is>
+          <t>협력사 (주)한영이엔씨 / 신호수 권복선 010-4506-6623 / 작업지휘자 차관종 010-5581-5199</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="8" t="n">
@@ -1459,5 +1607,6 @@
     <mergeCell ref="K3:L3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add forklift and aerial work platform rows to equipment ledger
Extract data from two more uploaded document sets: a hand-filled work
plan for a forklift (registration/model partly illegible, flagged with
comments) and a complete document set for a HS320 aerial work platform
(registration, inspection, insurance, operator license, business
registration).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011AyaoccyvsKxVgYNBrnxVL
</commit_message>
<xml_diff>
--- a/output/건설기계_기초자료_관리대장.xlsx
+++ b/output/건설기계_기초자료_관리대장.xlsx
@@ -259,6 +259,36 @@
     <comment ref="L6" authorId="0" shapeId="0">
       <text>
         <t>등록·검사증 뒷면 손글씨 기재분으로 판독이 어려워 추정 입력했습니다. 원본 서류로 반드시 재확인 바랍니다.</t>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0" shapeId="0">
+      <text>
+        <t>[건설기계의 종류] 체크박스가 '차량계 하역운반기계'+'중량물 취급'에 표시되어 있어 지게차로 추정했습니다.</t>
+      </text>
+    </comment>
+    <comment ref="C7" authorId="0" shapeId="0">
+      <text>
+        <t>모델명 손글씨(예: E70EV-9 유사)를 정확히 판독하지 못했습니다. 두산 지게차 정품 서류로 재확인 바랍니다.</t>
+      </text>
+    </comment>
+    <comment ref="D7" authorId="0" shapeId="0">
+      <text>
+        <t>등록번호 앞부분(지역+문자)이 정정선/필체로 가려져 있습니다. 뒷자리 '8206'만 확실합니다.</t>
+      </text>
+    </comment>
+    <comment ref="P7" authorId="0" shapeId="0">
+      <text>
+        <t>운전자 성명 손글씨(초서체)를 확정하지 못했습니다.</t>
+      </text>
+    </comment>
+    <comment ref="H8" authorId="0" shapeId="0">
+      <text>
+        <t>사업자등록증 상호는 '진스카이', 대표자 성명은 자동차등록증·보험증권 기준 '전은지'로 표기했습니다(사업자등록증 인쇄본의 성명 표기가 다소 흐려 재확인 권장).</t>
+      </text>
+    </comment>
+    <comment ref="J8" authorId="0" shapeId="0">
+      <text>
+        <t>소유자(전은지) 직통 연락처는 서류에서 마스킹/미기재되어 확인하지 못했습니다.</t>
       </text>
     </comment>
   </commentList>
@@ -975,53 +1005,219 @@
       <c r="A7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="9" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-      <c r="M7" s="8" t="n"/>
-      <c r="N7" s="8" t="n"/>
-      <c r="O7" s="8" t="n"/>
-      <c r="P7" s="8" t="n"/>
-      <c r="Q7" s="8" t="n"/>
-      <c r="R7" s="8" t="n"/>
-      <c r="S7" s="8" t="n"/>
-      <c r="T7" s="9" t="n"/>
-      <c r="U7" s="9" t="n"/>
-      <c r="V7" s="8" t="n"/>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>지게차</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>두산 / 7톤급 (모델명 필체 판독 어려움)</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>○○04○8206 (등록번호 필체 판독 어려움)</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>두산</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>010-6416-0540</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>정기검사</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>2023-10-16 ~ 2026-10-06</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>2025-10-2X ~ 2026-10-2X (일자 필체 판독 어려움)</t>
+        </is>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>판독 어려움(원본 확인 필요)</t>
+        </is>
+      </c>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t>건설기계조종사 면허 (세부 필체 판독 어려움)</t>
+        </is>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T7" s="9" t="inlineStr">
+        <is>
+          <t>현장내 (구체 현장명·공종 필체 판독 어려움)</t>
+        </is>
+      </c>
+      <c r="U7" s="8" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="V7" s="9" t="inlineStr">
+        <is>
+          <t>협력업체명·공종·작업내용·운전자 성명 등 손글씨 다수 판독 어려움 - 원본 대조 필요. 조종사안전교육수료 유 / 건설업기초안전보건교육 유. 정기검사·연락처는 인쇄체로 명확히 확인됨.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="8" t="n"/>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
-      <c r="L8" s="8" t="n"/>
-      <c r="M8" s="8" t="n"/>
-      <c r="N8" s="8" t="n"/>
-      <c r="O8" s="8" t="n"/>
-      <c r="P8" s="8" t="n"/>
-      <c r="Q8" s="8" t="n"/>
-      <c r="R8" s="8" t="n"/>
-      <c r="S8" s="8" t="n"/>
-      <c r="T8" s="9" t="n"/>
-      <c r="U8" s="9" t="n"/>
-      <c r="V8" s="8" t="n"/>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>고소작업대(차량탑재형)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>HS320(2018) / 3.5톤, 현대 3.5톤 장축슈퍼캡</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>전북98아2098</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>KMFHA17GPJC026862 (원동기형식 D4GB)</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>한신울트라</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>진스카이</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>전은지</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>정기검사</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>2025-09-21 ~ 2026-03-20</t>
+        </is>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>삼성화재해상보험(주)</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>125C4065440000</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>2025-02-13 ~ 2026-02-13</t>
+        </is>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>진상호</t>
+        </is>
+      </c>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>화물운송종사자격(1-14-171715) / 이동식크레인·고소작업대 조종교육 이수(2019-03-21)</t>
+        </is>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
+        <is>
+          <t>1-14-171715</t>
+        </is>
+      </c>
+      <c r="S8" s="8" t="inlineStr">
+        <is>
+          <t>자동차면허 적성검사 2027-01-01~2027-12-31 (화물자격 취득 2014-10-21)</t>
+        </is>
+      </c>
+      <c r="T8" s="9" t="inlineStr">
+        <is>
+          <t>본관동·후생동·경비동·신관동 (금속창호 - 각동 창호설치 및 유리작업)</t>
+        </is>
+      </c>
+      <c r="U8" s="8" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="V8" s="9" t="inlineStr">
+        <is>
+          <t>협력사 대호엔지니어링 / 작업지휘자 김남용 010-2756-4415 / 신호수 최하영 010-6202-9266</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="8" t="n">

</xml_diff>

<commit_message>
Add roller and mobile crane rows to equipment ledger
Extract data from two more uploaded document sets: a CAT CS54 roller
(registration, insurance, business registration) and a Dasan DTC-160
mobile crane (registration, insurance, operator license, NDT report).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011AyaoccyvsKxVgYNBrnxVL
</commit_message>
<xml_diff>
--- a/output/건설기계_기초자료_관리대장.xlsx
+++ b/output/건설기계_기초자료_관리대장.xlsx
@@ -289,6 +289,26 @@
     <comment ref="J8" authorId="0" shapeId="0">
       <text>
         <t>소유자(전은지) 직통 연락처는 서류에서 마스킹/미기재되어 확인하지 못했습니다.</t>
+      </text>
+    </comment>
+    <comment ref="G9" authorId="0" shapeId="0">
+      <text>
+        <t>등록·검사증에 '제작년도' 항목이 별도로 인쇄되어 있지 않아 확인하지 못했습니다(최초등록일 2011-12-29).</t>
+      </text>
+    </comment>
+    <comment ref="Q9" authorId="0" shapeId="0">
+      <text>
+        <t>면허종류가 롤러가 아닌 '굴착기'로 기재되어 있습니다(작업계획서 원문 그대로 옮김) - 실제 보유 면허 확인 필요.</t>
+      </text>
+    </comment>
+    <comment ref="V9" authorId="0" shapeId="0">
+      <text>
+        <t>신호수 성명 손글씨(방수경 추정)를 확정하지 못했습니다.</t>
+      </text>
+    </comment>
+    <comment ref="I10" authorId="0" shapeId="0">
+      <text>
+        <t>사업자등록증 인쇄상태가 흐려 대표자 성명이 '성상소'로도 보일 수 있으나, 조종면허증·안전교육이수증 등 다른 서류 3건에 모두 '정상조'로 표기되어 이를 채택했습니다.</t>
       </text>
     </comment>
   </commentList>
@@ -1223,53 +1243,219 @@
       <c r="A9" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="9" t="n"/>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8" t="n"/>
-      <c r="K9" s="8" t="n"/>
-      <c r="L9" s="8" t="n"/>
-      <c r="M9" s="8" t="n"/>
-      <c r="N9" s="8" t="n"/>
-      <c r="O9" s="8" t="n"/>
-      <c r="P9" s="8" t="n"/>
-      <c r="Q9" s="8" t="n"/>
-      <c r="R9" s="8" t="n"/>
-      <c r="S9" s="8" t="n"/>
-      <c r="T9" s="9" t="n"/>
-      <c r="U9" s="9" t="n"/>
-      <c r="V9" s="8" t="n"/>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>롤러</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>CS54 / 10.8톤</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>전북09바5460</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>CATOCS54TC5W00522</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>동아포장중기</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>김남의</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>010-3676-2675</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>정기검사</t>
+        </is>
+      </c>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>2023-12-26 ~ 2026-12-28</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>삼성화재해상보험(주)</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>125F0428890000</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>2025-03-23 ~ 2026-03-23</t>
+        </is>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>김남의</t>
+        </is>
+      </c>
+      <c r="Q9" s="8" t="inlineStr">
+        <is>
+          <t>굴착기(건설기계조종사)</t>
+        </is>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S9" s="8" t="inlineStr">
+        <is>
+          <t>2002-08-19 취득 (조종사 안전교육 별도 확인 필요)</t>
+        </is>
+      </c>
+      <c r="T9" s="9" t="inlineStr">
+        <is>
+          <t>현장내 도로 부지 (조풍건설 - 포장공사, 잡석 및 보조기층 다짐)</t>
+        </is>
+      </c>
+      <c r="U9" s="8" t="inlineStr">
+        <is>
+          <t>2025-11-12</t>
+        </is>
+      </c>
+      <c r="V9" s="9" t="inlineStr">
+        <is>
+          <t>협력업체 조풍건설 / 작업지휘자 오인석 010-9453-2038 / 신호수 방수경(추정) 010-4652-4457</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="8" t="n"/>
-      <c r="J10" s="8" t="n"/>
-      <c r="K10" s="8" t="n"/>
-      <c r="L10" s="8" t="n"/>
-      <c r="M10" s="8" t="n"/>
-      <c r="N10" s="8" t="n"/>
-      <c r="O10" s="8" t="n"/>
-      <c r="P10" s="8" t="n"/>
-      <c r="Q10" s="8" t="n"/>
-      <c r="R10" s="8" t="n"/>
-      <c r="S10" s="8" t="n"/>
-      <c r="T10" s="9" t="n"/>
-      <c r="U10" s="9" t="n"/>
-      <c r="V10" s="8" t="n"/>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>이동식크레인</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>DTC-160 / 16.37톤</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>007가9298</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>KLTLC3AH9GK000002 (원동기형식 F4AFE611C)</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>다산중공업</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>성상크레인</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>정상조</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>010-8874-7175</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>정기검사</t>
+        </is>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>2024-12-20 ~ 2026-01-09</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>삼성화재해상보험(주)</t>
+        </is>
+      </c>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>125M3774240000</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>2025-06-23 ~ 2026-06-23</t>
+        </is>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>정상조</t>
+        </is>
+      </c>
+      <c r="Q10" s="8" t="inlineStr">
+        <is>
+          <t>건설기계조종사(기중기)</t>
+        </is>
+      </c>
+      <c r="R10" s="8" t="inlineStr">
+        <is>
+          <t>경기20-2021-0646-00</t>
+        </is>
+      </c>
+      <c r="S10" s="8" t="inlineStr">
+        <is>
+          <t>2031-12-31(안전교육/적성검사 기준, 취득 2021-07-09)</t>
+        </is>
+      </c>
+      <c r="T10" s="9" t="inlineStr">
+        <is>
+          <t>부품창고동·본관동·후생동 (신우산업 - 판넬공사, 판넬설치·하지설치)</t>
+        </is>
+      </c>
+      <c r="U10" s="8" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="V10" s="9" t="inlineStr">
+        <is>
+          <t>협력업체 신우산업 / 작업지휘자 김상혁 010-4841-8713 / 신호수 강재구 010-2624-2670 / 비파괴검사(자분탐상, ICME 2025-10-21) Hook·Boom·Cylinder·TurnTable·Outrigger 전부 이상없음</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="n">

</xml_diff>